<commit_message>
feat: actualizaciones backend y frontend
</commit_message>
<xml_diff>
--- a/backend/plantillas/plantilla_asignaturas_ras.xlsx
+++ b/backend/plantillas/plantilla_asignaturas_ras.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asignaturas y RAs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,10 +444,15 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>sede</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>ra_descripcion</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>ra_porcentaje</t>
         </is>
@@ -456,106 +461,41 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ING101</t>
+          <t>750026C</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Introducción a Ingeniería</t>
+          <t>DESARROLLO DE APLICACIONES PARA DISPOSITIVOS MOVILES</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DOC001</t>
+          <t>DOC1001</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>INGSIS</t>
+          <t>2724</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>50</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Aplicar conceptos básicos de ingeniería</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>ING101</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Introducción a Ingeniería</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>DOC001</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>INGSIS</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Trabajar en equipo efectivamente</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>ING101</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Introducción a Ingeniería</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>DOC001</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>INGSIS</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Comunicar ideas técnicas</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>25</v>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Construye aplicaciones moviles funcionales</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: ajustes de importacion y vistas de coordinador
</commit_message>
<xml_diff>
--- a/backend/plantillas/plantilla_asignaturas_ras.xlsx
+++ b/backend/plantillas/plantilla_asignaturas_ras.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,20 +439,30 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>periodo</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>grupo</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>sede</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>creditos</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
         <is>
           <t>ra_descripcion</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>ra_porcentaje</t>
         </is>
@@ -479,22 +489,24 @@
           <t>2724</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>02</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
         <is>
           <t>Construye aplicaciones moviles funcionales</t>
         </is>
       </c>
-      <c r="H2" t="n">
+      <c r="J2" t="n">
         <v>50</v>
       </c>
     </row>

</xml_diff>